<commit_message>
Change RADME file, fix errors in main.py and add interactions with store.xlsx file. Also .gitignore was added
</commit_message>
<xml_diff>
--- a/store.xlsx
+++ b/store.xlsx
@@ -98,6 +98,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -390,51 +391,51 @@
         <v>14</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>400</v>
+        <v>10</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="0" t="n">
-        <v>200</v>
-      </c>
-      <c r="D3" s="0" t="n">
+      <c r="C3" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="D3" s="1" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="0" t="n">
-        <v>600</v>
-      </c>
-      <c r="D4" s="0" t="n">
+      <c r="C4" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="D4" s="1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="0" t="n">
-        <v>300</v>
-      </c>
-      <c r="D5" s="0" t="n">
+      <c r="C5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="1" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>